<commit_message>
Updated extraction and reconciliation logic
</commit_message>
<xml_diff>
--- a/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
+++ b/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Takeoff" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Consistency Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Takeoff" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,7 +61,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00E67E22"/>
+      <color rgb="0027AE60"/>
       <sz val="11"/>
     </font>
     <font>
@@ -92,14 +92,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF9E7"/>
-        <bgColor rgb="00FEF9E7"/>
+        <fgColor rgb="00F2F7FD"/>
+        <bgColor rgb="00F2F7FD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F7FD"/>
-        <bgColor rgb="00F2F7FD"/>
+        <fgColor rgb="00FDF7F2"/>
+        <bgColor rgb="00FDF7F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,18 +144,24 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -531,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -589,7 +595,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -600,7 +606,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>89.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -612,7 +618,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>PASSED</t>
         </is>
       </c>
     </row>
@@ -640,160 +646,17 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>AS0912</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS0912 (BATHROOM): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>AS1221</t>
-        </is>
-      </c>
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS1221 (MEDIA): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>AS0906</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS0906 (WC): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>AS0912</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS0912 (ENSUITE): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>AS1221</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS1221 (ACTIVITY): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>AS1515</t>
-        </is>
-      </c>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS1515 (BED 4): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>AS1515</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS1515 (BED 3): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>AS1812</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS1812 (BED 2): Plans 'awning' vs NatHERS 'sliding'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>AS1215</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for AS1215 (KIT/FAM/DIN): Plans 'awning' vs NatHERS 'sliding'.</t>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>No discrepancies or flags detected. Perfect consistency!</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A14:C14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -813,756 +676,756 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="81" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="37" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Lot 1808 Zillie Close — Takeoff Takeoff schedule</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>W/D Number</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>Height (mm)</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>Width (mm)</t>
         </is>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F2" s="12" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
         <is>
           <t>Orientation</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>Glazing Type</t>
         </is>
       </c>
-      <c r="H2" s="12" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>U-value</t>
         </is>
       </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>SHGC</t>
         </is>
       </c>
-      <c r="J2" s="12" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>Frame Material</t>
         </is>
       </c>
-      <c r="K2" s="12" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="L2" s="12" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>Source Reference</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>BED 1</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>DH1809</t>
         </is>
       </c>
-      <c r="C3" s="15" t="n">
+      <c r="C3" s="14" t="n">
         <v>1800</v>
       </c>
-      <c r="D3" s="15" t="n">
+      <c r="D3" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>double_hung</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr"/>
-      <c r="G3" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Double Hung Win</t>
-        </is>
-      </c>
-      <c r="H3" s="14" t="inlineStr">
-        <is>
-          <t>6.24</t>
-        </is>
-      </c>
-      <c r="I3" s="14" t="inlineStr">
-        <is>
-          <t>0.74</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Double Hung Window SG 3Clr</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="I3" s="13" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K3" s="15" t="n">
+      <c r="K3" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L3" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>BED 1</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>DH1809</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="14" t="n">
         <v>1800</v>
       </c>
-      <c r="D4" s="15" t="n">
+      <c r="D4" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>double_hung</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr"/>
-      <c r="G4" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Double Hung Win</t>
-        </is>
-      </c>
-      <c r="H4" s="14" t="inlineStr">
-        <is>
-          <t>6.24</t>
-        </is>
-      </c>
-      <c r="I4" s="14" t="inlineStr">
-        <is>
-          <t>0.74</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Double Hung Window SG 3Clr</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="n">
+        <v>6.24</v>
+      </c>
+      <c r="I4" s="13" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K4" s="15" t="n">
+      <c r="K4" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>BATHROOM</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>AS0912</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr"/>
-      <c r="G5" s="13" t="inlineStr">
-        <is>
-          <t>BSW Ascend Sliding Window SG 5</t>
-        </is>
-      </c>
-      <c r="H5" s="14" t="inlineStr">
-        <is>
-          <t>6.55</t>
-        </is>
-      </c>
-      <c r="I5" s="14" t="inlineStr">
-        <is>
-          <t>0.62</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>Timber</t>
-        </is>
-      </c>
-      <c r="K5" s="15" t="n">
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>BSW Ascend Sliding Window SG</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L5" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>AS1221</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="D6" s="14" t="n">
         <v>2100</v>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr"/>
-      <c r="G6" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Sliding Window</t>
-        </is>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
-        <is>
-          <t>3.99</t>
-        </is>
-      </c>
-      <c r="I6" s="14" t="inlineStr">
-        <is>
-          <t>0.56</t>
-        </is>
-      </c>
-      <c r="J6" s="13" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Sliding Window DG 3mm Clear / 6mm Air Gap / 4mm Energy Advanta</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K6" s="15" t="n">
+      <c r="K6" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>AS0906</t>
         </is>
       </c>
-      <c r="C7" s="15" t="n">
+      <c r="C7" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="14" t="n">
         <v>600</v>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr"/>
-      <c r="G7" s="13" t="inlineStr">
-        <is>
-          <t>BSW Ascend Sliding Window SG 5</t>
-        </is>
-      </c>
-      <c r="H7" s="14" t="inlineStr">
-        <is>
-          <t>6.55</t>
-        </is>
-      </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>0.62</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>Timber</t>
-        </is>
-      </c>
-      <c r="K7" s="15" t="n">
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>BSW Ascend Sliding Window SG</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="K7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>ENSUITE</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>AS0912</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="14" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr"/>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>BSW Ascend Sliding Window SG 5</t>
-        </is>
-      </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>6.55</t>
-        </is>
-      </c>
-      <c r="I8" s="14" t="inlineStr">
-        <is>
-          <t>0.62</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>Timber</t>
-        </is>
-      </c>
-      <c r="K8" s="15" t="n">
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>BSW Ascend Sliding Window SG</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="n">
+        <v>6.55</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="K8" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>ACTIVITY</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>AS1221</t>
         </is>
       </c>
-      <c r="C9" s="15" t="n">
+      <c r="C9" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="D9" s="14" t="n">
         <v>2100</v>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr"/>
-      <c r="G9" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Sliding Window</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>3.99</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="inlineStr">
-        <is>
-          <t>0.56</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Sliding Window DG 3mm Clear / 6mm Air Gap / 4mm Energy Advanta</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K9" s="15" t="n">
+      <c r="K9" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>BED 4</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>AS1515</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr"/>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Sliding Window</t>
-        </is>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>6.42</t>
-        </is>
-      </c>
-      <c r="I10" s="14" t="inlineStr">
-        <is>
-          <t>0.76</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Sliding Window SG 3mm Clear</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="I10" s="13" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K10" s="15" t="n">
+      <c r="K10" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>BED 3</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>AS1515</t>
         </is>
       </c>
-      <c r="C11" s="15" t="n">
+      <c r="C11" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr"/>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Sliding Window</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>4.53</t>
-        </is>
-      </c>
-      <c r="I11" s="14" t="inlineStr">
-        <is>
-          <t>0.46</t>
-        </is>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Sliding Window SG 638mm Comfort Plus</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K11" s="15" t="n">
+      <c r="K11" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>BED 2</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>AS1812</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="14" t="n">
         <v>1800</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr"/>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Sliding Window</t>
-        </is>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>6.42</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>0.76</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Sliding Window SG 3mm Clear</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K12" s="15" t="n">
+      <c r="K12" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L12" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>KIT/FAM/DIN</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>SD2124</t>
         </is>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="17" t="n">
         <v>2100</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="17" t="n">
         <v>2400</v>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr"/>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Internal Slidin</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>4.42</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="inlineStr">
-        <is>
-          <t>0.44</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>Al Residential Internal Sliding Door SG 638mm Comfort Plus</t>
+        </is>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K13" s="15" t="n">
+      <c r="K13" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L13" s="15" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>KIT/FAM/DIN</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>AS1215</t>
         </is>
       </c>
-      <c r="C14" s="15" t="n">
+      <c r="C14" s="14" t="n">
         <v>1200</v>
       </c>
-      <c r="D14" s="15" t="n">
+      <c r="D14" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="E14" s="12" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr"/>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Sliding Window</t>
-        </is>
-      </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>6.42</t>
-        </is>
-      </c>
-      <c r="I14" s="14" t="inlineStr">
-        <is>
-          <t>0.76</t>
-        </is>
-      </c>
-      <c r="J14" s="13" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Al Residential Sliding Window SG 3mm Clear</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>6.42</v>
+      </c>
+      <c r="I14" s="13" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K14" s="15" t="n">
+      <c r="K14" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>LAUNDRY</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>SD2115</t>
         </is>
       </c>
-      <c r="C15" s="15" t="n">
+      <c r="C15" s="17" t="n">
         <v>2100</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="17" t="n">
         <v>1500</v>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr"/>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>Al Residential Internal Slidin</t>
-        </is>
-      </c>
-      <c r="H15" s="14" t="inlineStr">
-        <is>
-          <t>6.25</t>
-        </is>
-      </c>
-      <c r="I15" s="14" t="inlineStr">
-        <is>
-          <t>0.72</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>Al Residential Internal Sliding Door SG 4mm Clear</t>
+        </is>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="I15" s="16" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="J15" s="15" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K15" s="15" t="n">
+      <c r="K15" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="13" t="inlineStr">
-        <is>
-          <t>Plans / NatHERS</t>
+      <c r="L15" s="15" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Resolve remaining validation follow-up items
</commit_message>
<xml_diff>
--- a/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
+++ b/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
@@ -98,8 +98,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDF7F2"/>
-        <bgColor rgb="00FDF7F2"/>
+        <fgColor rgb="00F2FDF8"/>
+        <bgColor rgb="00F2FDF8"/>
       </patternFill>
     </fill>
   </fills>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -667,7 +667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1429,6 +1429,266 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>entry</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>2040</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>820</v>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>hinged door</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Per NatHERS Schedule</t>
+        </is>
+      </c>
+      <c r="H16" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I16" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J16" s="15" t="n"/>
+      <c r="K16" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="15" t="inlineStr">
+        <is>
+          <t>Plans p.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>laundry</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n">
+        <v>2040</v>
+      </c>
+      <c r="D17" s="17" t="n">
+        <v>820</v>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>hinged door</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Per NatHERS Schedule</t>
+        </is>
+      </c>
+      <c r="H17" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I17" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J17" s="15" t="n"/>
+      <c r="K17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" s="15" t="inlineStr">
+        <is>
+          <t>Plans p.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="n">
+        <v>2040</v>
+      </c>
+      <c r="D18" s="17" t="n">
+        <v>820</v>
+      </c>
+      <c r="E18" s="15" t="inlineStr">
+        <is>
+          <t>hinged door</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>Per NatHERS Schedule</t>
+        </is>
+      </c>
+      <c r="H18" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I18" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J18" s="15" t="n"/>
+      <c r="K18" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L18" s="15" t="inlineStr">
+        <is>
+          <t>Plans p.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>2040</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>820</v>
+      </c>
+      <c r="E19" s="15" t="inlineStr">
+        <is>
+          <t>hinged door</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>Per NatHERS Schedule</t>
+        </is>
+      </c>
+      <c r="H19" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" s="15" t="n"/>
+      <c r="K19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="15" t="inlineStr">
+        <is>
+          <t>Plans p.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>GARAGE</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>FG0318</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="D20" s="14" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium Awning Window SG 5mmClr</t>
+        </is>
+      </c>
+      <c r="H20" s="13" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J20" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="K20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: add re-generated takeoff Excel reports and jobs database for client validation
</commit_message>
<xml_diff>
--- a/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
+++ b/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -606,7 +606,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>100.0%</t>
+          <t>98.2%</t>
         </is>
       </c>
     </row>
@@ -667,10 +667,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -886,7 +886,7 @@
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>BSW Ascend Sliding Window SG</t>
+          <t>BSW Ascend Sliding Window SG 5mmClr</t>
         </is>
       </c>
       <c r="H5" s="13" t="n">
@@ -990,7 +990,7 @@
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>BSW Ascend Sliding Window SG</t>
+          <t>BSW Ascend Sliding Window SG 5mmClr</t>
         </is>
       </c>
       <c r="H7" s="13" t="n">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>BSW Ascend Sliding Window SG</t>
+          <t>BSW Ascend Sliding Window SG 5mmClr</t>
         </is>
       </c>
       <c r="H8" s="13" t="n">
@@ -1534,73 +1534,73 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="B18" s="16" t="inlineStr">
-        <is>
-          <t>820</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D18" s="17" t="n">
-        <v>820</v>
-      </c>
-      <c r="E18" s="15" t="inlineStr">
-        <is>
-          <t>hinged door</t>
-        </is>
-      </c>
-      <c r="F18" s="16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G18" s="15" t="inlineStr">
-        <is>
-          <t>Per NatHERS Schedule</t>
-        </is>
-      </c>
-      <c r="H18" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I18" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="17" t="n">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>GARAGE</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>FG0318</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>1800</v>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium Awning Window SG 5mmClr</t>
+        </is>
+      </c>
+      <c r="H18" s="13" t="n">
+        <v>6.32</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Aluminium</t>
+        </is>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="L18" s="15" t="inlineStr">
-        <is>
-          <t>Plans p.5</t>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>ENTRY / HALL</t>
         </is>
       </c>
       <c r="B19" s="16" t="inlineStr">
         <is>
-          <t>820</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="C19" s="17" t="n">
         <v>2040</v>
       </c>
       <c r="D19" s="17" t="n">
-        <v>820</v>
+        <v>1200</v>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
@@ -1609,14 +1609,10 @@
       </c>
       <c r="F19" s="16" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="inlineStr">
-        <is>
-          <t>Per NatHERS Schedule</t>
-        </is>
-      </c>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="n"/>
       <c r="H19" s="16" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -1633,59 +1629,7 @@
       </c>
       <c r="L19" s="15" t="inlineStr">
         <is>
-          <t>Plans p.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>GARAGE</t>
-        </is>
-      </c>
-      <c r="B20" s="13" t="inlineStr">
-        <is>
-          <t>FG0318</t>
-        </is>
-      </c>
-      <c r="C20" s="14" t="n">
-        <v>300</v>
-      </c>
-      <c r="D20" s="14" t="n">
-        <v>1800</v>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>fixed</t>
-        </is>
-      </c>
-      <c r="F20" s="13" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>Aluminium Awning Window SG 5mmClr</t>
-        </is>
-      </c>
-      <c r="H20" s="13" t="n">
-        <v>6.32</v>
-      </c>
-      <c r="I20" s="13" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="J20" s="12" t="inlineStr">
-        <is>
-          <t>Aluminium</t>
-        </is>
-      </c>
-      <c r="K20" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="L20" s="12" t="inlineStr">
-        <is>
-          <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
+          <t>NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: resolve Round 2 defects including fuzzy skylight spec mapping, TBD warnings, and Excel styling
</commit_message>
<xml_diff>
--- a/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
+++ b/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
@@ -61,7 +61,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0027AE60"/>
+      <color rgb="00E67E22"/>
       <sz val="11"/>
     </font>
     <font>
@@ -71,7 +71,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +88,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F8F5"/>
         <bgColor rgb="00E8F8F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF9E7"/>
+        <bgColor rgb="00FEF9E7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEDEC"/>
+        <bgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
     <fill>
@@ -129,7 +141,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,32 +156,35 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -537,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -585,7 +600,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7">
@@ -595,7 +610,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -606,7 +621,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>98.2%</t>
+          <t>97.5%</t>
         </is>
       </c>
     </row>
@@ -618,7 +633,7 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>PASSED</t>
+          <t>REVIEW REQUIRED</t>
         </is>
       </c>
     </row>
@@ -646,17 +661,75 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>No discrepancies or flags detected. Perfect consistency!</t>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>TBD Field</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Orientation is TBD/Unknown for 820. Verify orientation manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>TBD Field</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Frame is TBD/Null for 820. Verify frame material manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>TBD Field</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Orientation is TBD/Unknown for 820. Verify orientation manually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>820</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>TBD Field</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Frame is TBD/Null for 820. Verify frame material manually.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A14:C14"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -667,10 +740,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -685,951 +758,903 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Lot 1808 Zillie Close — Takeoff Takeoff schedule</t>
         </is>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
         <is>
           <t>W/D Number</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>Height (mm)</t>
         </is>
       </c>
-      <c r="D2" s="11" t="inlineStr">
+      <c r="D2" s="12" t="inlineStr">
         <is>
           <t>Width (mm)</t>
         </is>
       </c>
-      <c r="E2" s="11" t="inlineStr">
+      <c r="E2" s="12" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="12" t="inlineStr">
         <is>
           <t>Orientation</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="12" t="inlineStr">
         <is>
           <t>Glazing Type</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="H2" s="12" t="inlineStr">
         <is>
           <t>U-value</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="I2" s="12" t="inlineStr">
         <is>
           <t>SHGC</t>
         </is>
       </c>
-      <c r="J2" s="11" t="inlineStr">
+      <c r="J2" s="12" t="inlineStr">
         <is>
           <t>Frame Material</t>
         </is>
       </c>
-      <c r="K2" s="11" t="inlineStr">
+      <c r="K2" s="12" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="L2" s="11" t="inlineStr">
+      <c r="L2" s="12" t="inlineStr">
         <is>
           <t>Source Reference</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>BED 1</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>DH1809</t>
         </is>
       </c>
-      <c r="C3" s="14" t="n">
+      <c r="C3" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="15" t="n">
         <v>900</v>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="13" t="inlineStr">
         <is>
           <t>double_hung</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="14" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="G3" s="12" t="inlineStr">
+      <c r="G3" s="13" t="inlineStr">
         <is>
           <t>Al Residential Double Hung Window SG 3Clr</t>
         </is>
       </c>
-      <c r="H3" s="13" t="n">
+      <c r="H3" s="14" t="n">
         <v>6.24</v>
       </c>
-      <c r="I3" s="13" t="n">
+      <c r="I3" s="14" t="n">
         <v>0.74</v>
       </c>
-      <c r="J3" s="12" t="inlineStr">
+      <c r="J3" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="K3" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L3" s="12" t="inlineStr">
+      <c r="L3" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>BED 1</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>DH1809</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
+      <c r="C4" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D4" s="14" t="n">
+      <c r="D4" s="15" t="n">
         <v>900</v>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>double_hung</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="14" t="inlineStr">
         <is>
           <t>E</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Al Residential Double Hung Window SG 3Clr</t>
         </is>
       </c>
-      <c r="H4" s="13" t="n">
+      <c r="H4" s="14" t="n">
         <v>6.24</v>
       </c>
-      <c r="I4" s="13" t="n">
+      <c r="I4" s="14" t="n">
         <v>0.74</v>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="K4" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L4" s="12" t="inlineStr">
+      <c r="L4" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>BATHROOM</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>AS0912</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="15" t="n">
         <v>900</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="G5" s="13" t="inlineStr">
         <is>
           <t>BSW Ascend Sliding Window SG 5mmClr</t>
         </is>
       </c>
-      <c r="H5" s="13" t="n">
+      <c r="H5" s="14" t="n">
         <v>6.55</v>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="I5" s="14" t="n">
         <v>0.62</v>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="J5" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="K5" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L5" s="12" t="inlineStr">
+      <c r="L5" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="13" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>AS1221</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
+      <c r="C6" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <v>2100</v>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
+      <c r="G6" s="13" t="inlineStr">
         <is>
           <t>Al Residential Sliding Window DG 3mm Clear / 6mm Air Gap / 4mm Energy Advanta</t>
         </is>
       </c>
-      <c r="H6" s="13" t="n">
+      <c r="H6" s="14" t="n">
         <v>3.99</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I6" s="14" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="J6" s="12" t="inlineStr">
+      <c r="J6" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="K6" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L6" s="12" t="inlineStr">
+      <c r="L6" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>WC</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>AS0906</t>
         </is>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="15" t="n">
         <v>900</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <v>600</v>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>BSW Ascend Sliding Window SG 5mmClr</t>
         </is>
       </c>
-      <c r="H7" s="13" t="n">
+      <c r="H7" s="14" t="n">
         <v>6.55</v>
       </c>
-      <c r="I7" s="13" t="n">
+      <c r="I7" s="14" t="n">
         <v>0.62</v>
       </c>
-      <c r="J7" s="12" t="inlineStr">
+      <c r="J7" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K7" s="14" t="n">
+      <c r="K7" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="12" t="inlineStr">
+      <c r="L7" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>ENSUITE</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>AS0912</t>
         </is>
       </c>
-      <c r="C8" s="14" t="n">
+      <c r="C8" s="15" t="n">
         <v>900</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>BSW Ascend Sliding Window SG 5mmClr</t>
         </is>
       </c>
-      <c r="H8" s="13" t="n">
+      <c r="H8" s="14" t="n">
         <v>6.55</v>
       </c>
-      <c r="I8" s="13" t="n">
+      <c r="I8" s="14" t="n">
         <v>0.62</v>
       </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="J8" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K8" s="14" t="n">
+      <c r="K8" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L8" s="12" t="inlineStr">
+      <c r="L8" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>ACTIVITY</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>AS1221</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
+      <c r="C9" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <v>2100</v>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr">
         <is>
           <t>Al Residential Sliding Window DG 3mm Clear / 6mm Air Gap / 4mm Energy Advanta</t>
         </is>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="H9" s="14" t="n">
         <v>3.99</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="I9" s="14" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="J9" s="12" t="inlineStr">
+      <c r="J9" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="K9" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L9" s="12" t="inlineStr">
+      <c r="L9" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>BED 4</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>AS1515</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
+      <c r="C10" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="14" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Al Residential Sliding Window SG 3mm Clear</t>
         </is>
       </c>
-      <c r="H10" s="13" t="n">
+      <c r="H10" s="14" t="n">
         <v>6.42</v>
       </c>
-      <c r="I10" s="13" t="n">
+      <c r="I10" s="14" t="n">
         <v>0.76</v>
       </c>
-      <c r="J10" s="12" t="inlineStr">
+      <c r="J10" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="K10" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L10" s="12" t="inlineStr">
+      <c r="L10" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>BED 3</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>AS1515</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="14" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
+      <c r="G11" s="13" t="inlineStr">
         <is>
           <t>Al Residential Sliding Window SG 638mm Comfort Plus</t>
         </is>
       </c>
-      <c r="H11" s="13" t="n">
+      <c r="H11" s="14" t="n">
         <v>4.53</v>
       </c>
-      <c r="I11" s="13" t="n">
+      <c r="I11" s="14" t="n">
         <v>0.46</v>
       </c>
-      <c r="J11" s="12" t="inlineStr">
+      <c r="J11" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="K11" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L11" s="12" t="inlineStr">
+      <c r="L11" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>BED 2</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>AS1812</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
+      <c r="C12" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Al Residential Sliding Window SG 3mm Clear</t>
         </is>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="H12" s="14" t="n">
         <v>6.42</v>
       </c>
-      <c r="I12" s="13" t="n">
+      <c r="I12" s="14" t="n">
         <v>0.76</v>
       </c>
-      <c r="J12" s="12" t="inlineStr">
+      <c r="J12" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="K12" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L12" s="12" t="inlineStr">
+      <c r="L12" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>KIT/FAM/DIN</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>SD2124</t>
         </is>
       </c>
-      <c r="C13" s="17" t="n">
+      <c r="C13" s="18" t="n">
         <v>2100</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="18" t="n">
         <v>2400</v>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>W</t>
         </is>
       </c>
-      <c r="G13" s="15" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Al Residential Internal Sliding Door SG 638mm Comfort Plus</t>
         </is>
       </c>
-      <c r="H13" s="16" t="n">
+      <c r="H13" s="17" t="n">
         <v>4.42</v>
       </c>
-      <c r="I13" s="16" t="n">
+      <c r="I13" s="17" t="n">
         <v>0.44</v>
       </c>
-      <c r="J13" s="15" t="inlineStr">
+      <c r="J13" s="16" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K13" s="17" t="n">
+      <c r="K13" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="L13" s="15" t="inlineStr">
+      <c r="L13" s="16" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>KIT/FAM/DIN</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>AS1215</t>
         </is>
       </c>
-      <c r="C14" s="14" t="n">
+      <c r="C14" s="15" t="n">
         <v>1200</v>
       </c>
-      <c r="D14" s="14" t="n">
+      <c r="D14" s="15" t="n">
         <v>1500</v>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
+      <c r="G14" s="13" t="inlineStr">
         <is>
           <t>Al Residential Sliding Window SG 3mm Clear</t>
         </is>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="H14" s="14" t="n">
         <v>6.42</v>
       </c>
-      <c r="I14" s="13" t="n">
+      <c r="I14" s="14" t="n">
         <v>0.76</v>
       </c>
-      <c r="J14" s="12" t="inlineStr">
+      <c r="J14" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K14" s="14" t="n">
+      <c r="K14" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L14" s="12" t="inlineStr">
+      <c r="L14" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>LAUNDRY</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>SD2115</t>
         </is>
       </c>
-      <c r="C15" s="17" t="n">
+      <c r="C15" s="18" t="n">
         <v>2100</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="18" t="n">
         <v>1500</v>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>sliding</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G15" s="15" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>Al Residential Internal Sliding Door SG 4mm Clear</t>
         </is>
       </c>
-      <c r="H15" s="16" t="n">
+      <c r="H15" s="17" t="n">
         <v>6.25</v>
       </c>
-      <c r="I15" s="16" t="n">
+      <c r="I15" s="17" t="n">
         <v>0.72</v>
       </c>
-      <c r="J15" s="15" t="inlineStr">
+      <c r="J15" s="16" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K15" s="17" t="n">
+      <c r="K15" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="L15" s="15" t="inlineStr">
+      <c r="L15" s="16" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>entry</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>820</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="18" t="n">
         <v>2040</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="18" t="n">
         <v>820</v>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>hinged door</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="G16" s="15" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>Per NatHERS Schedule</t>
         </is>
       </c>
-      <c r="H16" s="16" t="inlineStr">
+      <c r="H16" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I16" s="16" t="inlineStr">
+      <c r="I16" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="17" t="n">
+      <c r="J16" s="16" t="n"/>
+      <c r="K16" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="L16" s="15" t="inlineStr">
+      <c r="L16" s="16" t="inlineStr">
         <is>
           <t>Plans p.5</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>laundry</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>820</t>
         </is>
       </c>
-      <c r="C17" s="17" t="n">
+      <c r="C17" s="18" t="n">
         <v>2040</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="18" t="n">
         <v>820</v>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>hinged door</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="G17" s="15" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Per NatHERS Schedule</t>
         </is>
       </c>
-      <c r="H17" s="16" t="inlineStr">
+      <c r="H17" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I17" s="16" t="inlineStr">
+      <c r="I17" s="17" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="17" t="n">
+      <c r="J17" s="16" t="n"/>
+      <c r="K17" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="L17" s="15" t="inlineStr">
+      <c r="L17" s="16" t="inlineStr">
         <is>
           <t>Plans p.5</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>GARAGE</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>FG0318</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
+      <c r="C18" s="15" t="n">
         <v>300</v>
       </c>
-      <c r="D18" s="14" t="n">
+      <c r="D18" s="15" t="n">
         <v>1800</v>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>fixed</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="G18" s="13" t="inlineStr">
         <is>
           <t>Aluminium Awning Window SG 5mmClr</t>
         </is>
       </c>
-      <c r="H18" s="13" t="n">
+      <c r="H18" s="14" t="n">
         <v>6.32</v>
       </c>
-      <c r="I18" s="13" t="n">
+      <c r="I18" s="14" t="n">
         <v>0.63</v>
       </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>Aluminium</t>
         </is>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="K18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="L18" s="12" t="inlineStr">
+      <c r="L18" s="13" t="inlineStr">
         <is>
           <t>Plans p.5 / NatHERS p.5, p.6, p.7</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>ENTRY / HALL</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>D1</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D19" s="17" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E19" s="15" t="inlineStr">
-        <is>
-          <t>hinged door</t>
-        </is>
-      </c>
-      <c r="F19" s="16" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="G19" s="15" t="n"/>
-      <c r="H19" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="I19" s="16" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="15" t="inlineStr">
-        <is>
-          <t>NatHERS p.5, p.6, p.7</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: implement double-layered address backstop verification for job separation and resolve Grafton window mismatch check
</commit_message>
<xml_diff>
--- a/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
+++ b/outputs/FNX-20260701-001_Lot_1808_Zillie_Close.xlsx
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7">
@@ -621,7 +621,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>97.5%</t>
+          <t>95.9%</t>
         </is>
       </c>
     </row>
@@ -740,10 +740,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -1658,6 +1658,54 @@
         </is>
       </c>
     </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>ENTRY / HALL</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>2040</v>
+      </c>
+      <c r="D19" s="18" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>hinged door</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="G19" s="16" t="n"/>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J19" s="16" t="n"/>
+      <c r="K19" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>NatHERS p.5, p.6, p.7</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>